<commit_message>
Add Aug 25 practice GPS data to library
Clean CMJ season sheet already carried Aug 25 jump data; this adds the
matching Catapult export, converted to the library's minutes-based
Duration format used for per-minute calcs.
</commit_message>
<xml_diff>
--- a/sample_data/WSOC_CMJ_Season.xlsx
+++ b/sample_data/WSOC_CMJ_Season.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahc\Desktop\PLNU_WSOC_SS\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010BB5BA-65C0-4F9D-A83F-CF7F2E6556F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C50F9FF-9E33-45DC-9E3A-8C6C91C1E722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2835" yWindow="5070" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="33">
   <si>
     <t>Date</t>
   </si>
@@ -126,7 +126,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -182,7 +182,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,10 +485,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1382,6 +1383,467 @@
         <v>12.6</v>
       </c>
     </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B58" t="b">
+        <v>0</v>
+      </c>
+      <c r="C58" t="s">
+        <v>5</v>
+      </c>
+      <c r="D58">
+        <v>15.2</v>
+      </c>
+      <c r="E58">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B59" t="b">
+        <v>0</v>
+      </c>
+      <c r="C59" t="s">
+        <v>6</v>
+      </c>
+      <c r="D59">
+        <v>12.6</v>
+      </c>
+      <c r="E59">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B60" t="b">
+        <v>0</v>
+      </c>
+      <c r="C60" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60">
+        <v>14.6</v>
+      </c>
+      <c r="E60">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B61" t="b">
+        <v>0</v>
+      </c>
+      <c r="C61" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61">
+        <v>13.7</v>
+      </c>
+      <c r="E61">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B62" t="b">
+        <v>0</v>
+      </c>
+      <c r="C62" t="s">
+        <v>9</v>
+      </c>
+      <c r="D62">
+        <v>10.7</v>
+      </c>
+      <c r="E62">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B63" t="b">
+        <v>0</v>
+      </c>
+      <c r="C63" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B64" t="b">
+        <v>0</v>
+      </c>
+      <c r="C64" t="s">
+        <v>11</v>
+      </c>
+      <c r="D64">
+        <v>15.3</v>
+      </c>
+      <c r="E64">
+        <v>15.7</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B65" t="b">
+        <v>0</v>
+      </c>
+      <c r="C65" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65">
+        <v>10.6</v>
+      </c>
+      <c r="E65">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B66" t="b">
+        <v>0</v>
+      </c>
+      <c r="C66" t="s">
+        <v>13</v>
+      </c>
+      <c r="D66">
+        <v>13.7</v>
+      </c>
+      <c r="E66">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B67" t="b">
+        <v>0</v>
+      </c>
+      <c r="C67" t="s">
+        <v>14</v>
+      </c>
+      <c r="D67">
+        <v>12.8</v>
+      </c>
+      <c r="E67">
+        <v>12.9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B68" t="b">
+        <v>0</v>
+      </c>
+      <c r="C68" t="s">
+        <v>15</v>
+      </c>
+      <c r="D68">
+        <v>12.8</v>
+      </c>
+      <c r="E68">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B69" t="b">
+        <v>0</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>14.9</v>
+      </c>
+      <c r="E69">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B70" t="b">
+        <v>0</v>
+      </c>
+      <c r="C70" t="s">
+        <v>17</v>
+      </c>
+      <c r="D70">
+        <v>12.9</v>
+      </c>
+      <c r="E70">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B71" t="b">
+        <v>0</v>
+      </c>
+      <c r="C71" t="s">
+        <v>18</v>
+      </c>
+      <c r="D71">
+        <v>13.5</v>
+      </c>
+      <c r="E71">
+        <v>13.7</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B72" t="b">
+        <v>0</v>
+      </c>
+      <c r="C72" t="s">
+        <v>19</v>
+      </c>
+      <c r="D72">
+        <v>12.2</v>
+      </c>
+      <c r="E72">
+        <v>12.9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B73" t="b">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>20</v>
+      </c>
+      <c r="D73">
+        <v>12.8</v>
+      </c>
+      <c r="E73">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B74" t="b">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B75" t="b">
+        <v>0</v>
+      </c>
+      <c r="C75" t="s">
+        <v>22</v>
+      </c>
+      <c r="D75">
+        <v>11.6</v>
+      </c>
+      <c r="E75">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B76" t="b">
+        <v>0</v>
+      </c>
+      <c r="C76" t="s">
+        <v>23</v>
+      </c>
+      <c r="D76">
+        <v>14.9</v>
+      </c>
+      <c r="E76">
+        <v>15.2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B77" t="b">
+        <v>0</v>
+      </c>
+      <c r="C77" t="s">
+        <v>24</v>
+      </c>
+      <c r="D77">
+        <v>13.5</v>
+      </c>
+      <c r="E77">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B78" t="b">
+        <v>0</v>
+      </c>
+      <c r="C78" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B79" t="b">
+        <v>0</v>
+      </c>
+      <c r="C79" t="s">
+        <v>26</v>
+      </c>
+      <c r="D79">
+        <v>13.2</v>
+      </c>
+      <c r="E79">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B80" t="b">
+        <v>0</v>
+      </c>
+      <c r="C80" t="s">
+        <v>27</v>
+      </c>
+      <c r="D80">
+        <v>15.6</v>
+      </c>
+      <c r="E80">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B81" t="b">
+        <v>0</v>
+      </c>
+      <c r="C81" t="s">
+        <v>28</v>
+      </c>
+      <c r="D81">
+        <v>15.2</v>
+      </c>
+      <c r="E81">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B82" t="b">
+        <v>0</v>
+      </c>
+      <c r="C82" t="s">
+        <v>29</v>
+      </c>
+      <c r="D82">
+        <v>13.8</v>
+      </c>
+      <c r="E82">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B83" t="b">
+        <v>0</v>
+      </c>
+      <c r="C83" t="s">
+        <v>30</v>
+      </c>
+      <c r="D83">
+        <v>12.9</v>
+      </c>
+      <c r="E83">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B84" t="b">
+        <v>0</v>
+      </c>
+      <c r="C84" t="s">
+        <v>31</v>
+      </c>
+      <c r="D84">
+        <v>12.2</v>
+      </c>
+      <c r="E84">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B85" t="b">
+        <v>0</v>
+      </c>
+      <c r="C85" t="s">
+        <v>32</v>
+      </c>
+      <c r="D85">
+        <v>11.9</v>
+      </c>
+      <c r="E85">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Aug 31 CMJ testing data to the season sheet
Adds 28 rows for Monday Aug 31. Purely additive: the 84 existing rows
are unchanged, none dropped, columns unchanged, so no cleaning was
needed — the sheet already matches the schema the dashboard derives
from (Date / Match / Player Name / CMJ 1 / CMJ 2).

Validated: no duplicate player-per-date, roster stable at 28 across all
four dates, values 9.60-17.10 with no non-positive entries, and no
result more than 3 SD from that player's own prior history.

Dashboard now reports Monday, August 31 2026 as the testing date with
19 Green / 6 Yellow / 0 Red. The remaining 3 of 28 show No Data: Emma
Blakely and Madilyn Audet have still not recorded a jump this season,
and Kylee Jerome tested for the first time on Aug 31, so her rolling SD
is 0 and her Z-score is undefined until a second test.
</commit_message>
<xml_diff>
--- a/sample_data/WSOC_CMJ_Season.xlsx
+++ b/sample_data/WSOC_CMJ_Season.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahc\Desktop\PLNU_WSOC_SS\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C50F9FF-9E33-45DC-9E3A-8C6C91C1E722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86EC696A-D114-477C-97A9-F988F8CF24A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2835" yWindow="5070" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7155" yWindow="3900" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="33">
   <si>
     <t>Date</t>
   </si>
@@ -485,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E86"/>
+  <dimension ref="A1:E113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -1842,7 +1855,468 @@
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" s="2"/>
+      <c r="A86" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B86" t="b">
+        <v>0</v>
+      </c>
+      <c r="C86" t="s">
+        <v>5</v>
+      </c>
+      <c r="D86">
+        <v>16.5</v>
+      </c>
+      <c r="E86">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B87" t="b">
+        <v>0</v>
+      </c>
+      <c r="C87" t="s">
+        <v>6</v>
+      </c>
+      <c r="D87">
+        <v>13</v>
+      </c>
+      <c r="E87">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B88" t="b">
+        <v>0</v>
+      </c>
+      <c r="C88" t="s">
+        <v>7</v>
+      </c>
+      <c r="D88">
+        <v>15.5</v>
+      </c>
+      <c r="E88">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B89" t="b">
+        <v>0</v>
+      </c>
+      <c r="C89" t="s">
+        <v>8</v>
+      </c>
+      <c r="D89">
+        <v>12.7</v>
+      </c>
+      <c r="E89">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B90" t="b">
+        <v>0</v>
+      </c>
+      <c r="C90" t="s">
+        <v>9</v>
+      </c>
+      <c r="D90">
+        <v>11.4</v>
+      </c>
+      <c r="E90">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B91" t="b">
+        <v>0</v>
+      </c>
+      <c r="C91" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B92" t="b">
+        <v>0</v>
+      </c>
+      <c r="C92" t="s">
+        <v>11</v>
+      </c>
+      <c r="D92">
+        <v>14.4</v>
+      </c>
+      <c r="E92">
+        <v>15.2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B93" t="b">
+        <v>0</v>
+      </c>
+      <c r="C93" t="s">
+        <v>12</v>
+      </c>
+      <c r="D93">
+        <v>10.4</v>
+      </c>
+      <c r="E93">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B94" t="b">
+        <v>0</v>
+      </c>
+      <c r="C94" t="s">
+        <v>13</v>
+      </c>
+      <c r="D94">
+        <v>15.3</v>
+      </c>
+      <c r="E94">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B95" t="b">
+        <v>0</v>
+      </c>
+      <c r="C95" t="s">
+        <v>14</v>
+      </c>
+      <c r="D95">
+        <v>13.4</v>
+      </c>
+      <c r="E95">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B96" t="b">
+        <v>0</v>
+      </c>
+      <c r="C96" t="s">
+        <v>15</v>
+      </c>
+      <c r="D96">
+        <v>13</v>
+      </c>
+      <c r="E96">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B97" t="b">
+        <v>0</v>
+      </c>
+      <c r="C97" t="s">
+        <v>16</v>
+      </c>
+      <c r="D97">
+        <v>14.2</v>
+      </c>
+      <c r="E97">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B98" t="b">
+        <v>0</v>
+      </c>
+      <c r="C98" t="s">
+        <v>17</v>
+      </c>
+      <c r="D98">
+        <v>13.3</v>
+      </c>
+      <c r="E98">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B99" t="b">
+        <v>0</v>
+      </c>
+      <c r="C99" t="s">
+        <v>18</v>
+      </c>
+      <c r="D99">
+        <v>13.3</v>
+      </c>
+      <c r="E99">
+        <v>14.6</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B100" t="b">
+        <v>0</v>
+      </c>
+      <c r="C100" t="s">
+        <v>19</v>
+      </c>
+      <c r="D100">
+        <v>12.5</v>
+      </c>
+      <c r="E100">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B101" t="b">
+        <v>0</v>
+      </c>
+      <c r="C101" t="s">
+        <v>20</v>
+      </c>
+      <c r="D101">
+        <v>13</v>
+      </c>
+      <c r="E101">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B102" t="b">
+        <v>0</v>
+      </c>
+      <c r="C102" t="s">
+        <v>21</v>
+      </c>
+      <c r="D102">
+        <v>15.5</v>
+      </c>
+      <c r="E102">
+        <v>15.7</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B103" t="b">
+        <v>0</v>
+      </c>
+      <c r="C103" t="s">
+        <v>22</v>
+      </c>
+      <c r="D103">
+        <v>11.3</v>
+      </c>
+      <c r="E103">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B104" t="b">
+        <v>0</v>
+      </c>
+      <c r="C104" t="s">
+        <v>23</v>
+      </c>
+      <c r="D104">
+        <v>14</v>
+      </c>
+      <c r="E104">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B105" t="b">
+        <v>0</v>
+      </c>
+      <c r="C105" t="s">
+        <v>24</v>
+      </c>
+      <c r="D105">
+        <v>12.6</v>
+      </c>
+      <c r="E105">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B106" t="b">
+        <v>0</v>
+      </c>
+      <c r="C106" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B107" t="b">
+        <v>0</v>
+      </c>
+      <c r="C107" t="s">
+        <v>26</v>
+      </c>
+      <c r="D107">
+        <v>15.2</v>
+      </c>
+      <c r="E107">
+        <v>15.2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B108" t="b">
+        <v>0</v>
+      </c>
+      <c r="C108" t="s">
+        <v>27</v>
+      </c>
+      <c r="D108">
+        <v>15.4</v>
+      </c>
+      <c r="E108">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B109" t="b">
+        <v>0</v>
+      </c>
+      <c r="C109" t="s">
+        <v>28</v>
+      </c>
+      <c r="D109">
+        <v>17.100000000000001</v>
+      </c>
+      <c r="E109">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B110" t="b">
+        <v>0</v>
+      </c>
+      <c r="C110" t="s">
+        <v>29</v>
+      </c>
+      <c r="D110">
+        <v>12.6</v>
+      </c>
+      <c r="E110">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B111" t="b">
+        <v>0</v>
+      </c>
+      <c r="C111" t="s">
+        <v>30</v>
+      </c>
+      <c r="D111">
+        <v>13</v>
+      </c>
+      <c r="E111">
+        <v>12.9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B112" t="b">
+        <v>0</v>
+      </c>
+      <c r="C112" t="s">
+        <v>31</v>
+      </c>
+      <c r="D112">
+        <v>12.9</v>
+      </c>
+      <c r="E112">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A113" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B113" t="b">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>32</v>
+      </c>
+      <c r="D113">
+        <v>12.5</v>
+      </c>
+      <c r="E113">
+        <v>12.6</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Sep 8 CMJ data
Practice session, all 28 roster players. Beatrice Levi, Emma Blakely and
Grace Nelson have no jumps recorded; they carry through as blanks rather
than zeros, so their baselines and readiness stay untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/WSOC_CMJ_Season.xlsx
+++ b/sample_data/WSOC_CMJ_Season.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahc\Desktop\PLNU_WSOC_SS\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE7A5D79-6074-424D-B265-990C7680695E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39A234CB-3017-4C32-BC00-18EA622856BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1770" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="33">
   <si>
     <t>Date</t>
   </si>
@@ -498,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E253"/>
+  <dimension ref="A1:E281"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -4596,6 +4596,464 @@
         <v>11.7</v>
       </c>
     </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A254" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B254" t="b">
+        <v>0</v>
+      </c>
+      <c r="C254" t="s">
+        <v>5</v>
+      </c>
+      <c r="D254">
+        <v>14.2</v>
+      </c>
+      <c r="E254">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A255" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B255" t="b">
+        <v>0</v>
+      </c>
+      <c r="C255" t="s">
+        <v>6</v>
+      </c>
+      <c r="D255">
+        <v>13.9</v>
+      </c>
+      <c r="E255">
+        <v>13.7</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A256" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B256" t="b">
+        <v>0</v>
+      </c>
+      <c r="C256" t="s">
+        <v>7</v>
+      </c>
+      <c r="D256">
+        <v>13.9</v>
+      </c>
+      <c r="E256">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A257" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B257" t="b">
+        <v>0</v>
+      </c>
+      <c r="C257" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A258" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B258" t="b">
+        <v>0</v>
+      </c>
+      <c r="C258" t="s">
+        <v>9</v>
+      </c>
+      <c r="D258">
+        <v>11.3</v>
+      </c>
+      <c r="E258">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A259" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B259" t="b">
+        <v>0</v>
+      </c>
+      <c r="C259" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A260" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B260" t="b">
+        <v>0</v>
+      </c>
+      <c r="C260" t="s">
+        <v>11</v>
+      </c>
+      <c r="D260">
+        <v>15.1</v>
+      </c>
+      <c r="E260">
+        <v>15.2</v>
+      </c>
+    </row>
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A261" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B261" t="b">
+        <v>0</v>
+      </c>
+      <c r="C261" t="s">
+        <v>12</v>
+      </c>
+      <c r="D261">
+        <v>10.3</v>
+      </c>
+      <c r="E261">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A262" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B262" t="b">
+        <v>0</v>
+      </c>
+      <c r="C262" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A263" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B263" t="b">
+        <v>0</v>
+      </c>
+      <c r="C263" t="s">
+        <v>14</v>
+      </c>
+      <c r="D263">
+        <v>13.2</v>
+      </c>
+      <c r="E263">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A264" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B264" t="b">
+        <v>0</v>
+      </c>
+      <c r="C264" t="s">
+        <v>15</v>
+      </c>
+      <c r="D264">
+        <v>13.8</v>
+      </c>
+      <c r="E264">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A265" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B265" t="b">
+        <v>0</v>
+      </c>
+      <c r="C265" t="s">
+        <v>16</v>
+      </c>
+      <c r="D265">
+        <v>13.8</v>
+      </c>
+      <c r="E265">
+        <v>13.7</v>
+      </c>
+    </row>
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A266" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B266" t="b">
+        <v>0</v>
+      </c>
+      <c r="C266" t="s">
+        <v>17</v>
+      </c>
+      <c r="D266">
+        <v>13.3</v>
+      </c>
+      <c r="E266">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A267" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B267" t="b">
+        <v>0</v>
+      </c>
+      <c r="C267" t="s">
+        <v>18</v>
+      </c>
+      <c r="D267">
+        <v>14</v>
+      </c>
+      <c r="E267">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A268" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B268" t="b">
+        <v>0</v>
+      </c>
+      <c r="C268" t="s">
+        <v>19</v>
+      </c>
+      <c r="D268">
+        <v>10.9</v>
+      </c>
+      <c r="E268">
+        <v>9.6999999999999993</v>
+      </c>
+    </row>
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A269" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B269" t="b">
+        <v>0</v>
+      </c>
+      <c r="C269" t="s">
+        <v>20</v>
+      </c>
+      <c r="D269">
+        <v>13</v>
+      </c>
+      <c r="E269">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A270" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B270" t="b">
+        <v>0</v>
+      </c>
+      <c r="C270" t="s">
+        <v>21</v>
+      </c>
+      <c r="D270">
+        <v>15.4</v>
+      </c>
+      <c r="E270">
+        <v>15.7</v>
+      </c>
+    </row>
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A271" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B271" t="b">
+        <v>0</v>
+      </c>
+      <c r="C271" t="s">
+        <v>22</v>
+      </c>
+      <c r="D271">
+        <v>11.2</v>
+      </c>
+      <c r="E271">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A272" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B272" t="b">
+        <v>0</v>
+      </c>
+      <c r="C272" t="s">
+        <v>23</v>
+      </c>
+      <c r="D272">
+        <v>14.5</v>
+      </c>
+      <c r="E272">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A273" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B273" t="b">
+        <v>0</v>
+      </c>
+      <c r="C273" t="s">
+        <v>24</v>
+      </c>
+      <c r="D273">
+        <v>13.9</v>
+      </c>
+      <c r="E273">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A274" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B274" t="b">
+        <v>0</v>
+      </c>
+      <c r="C274" t="s">
+        <v>25</v>
+      </c>
+      <c r="D274">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="E274">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A275" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B275" t="b">
+        <v>0</v>
+      </c>
+      <c r="C275" t="s">
+        <v>26</v>
+      </c>
+      <c r="D275">
+        <v>13.4</v>
+      </c>
+      <c r="E275">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A276" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B276" t="b">
+        <v>0</v>
+      </c>
+      <c r="C276" t="s">
+        <v>27</v>
+      </c>
+      <c r="D276">
+        <v>15.4</v>
+      </c>
+      <c r="E276">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A277" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B277" t="b">
+        <v>0</v>
+      </c>
+      <c r="C277" t="s">
+        <v>28</v>
+      </c>
+      <c r="D277">
+        <v>16</v>
+      </c>
+      <c r="E277">
+        <v>15.9</v>
+      </c>
+    </row>
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A278" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B278" t="b">
+        <v>0</v>
+      </c>
+      <c r="C278" t="s">
+        <v>29</v>
+      </c>
+      <c r="D278">
+        <v>13.6</v>
+      </c>
+      <c r="E278">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A279" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B279" t="b">
+        <v>0</v>
+      </c>
+      <c r="C279" t="s">
+        <v>30</v>
+      </c>
+      <c r="D279">
+        <v>12.4</v>
+      </c>
+      <c r="E279">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A280" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B280" t="b">
+        <v>0</v>
+      </c>
+      <c r="C280" t="s">
+        <v>31</v>
+      </c>
+      <c r="D280">
+        <v>13</v>
+      </c>
+      <c r="E280">
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A281" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B281" t="b">
+        <v>0</v>
+      </c>
+      <c r="C281" t="s">
+        <v>32</v>
+      </c>
+      <c r="D281">
+        <v>11.6</v>
+      </c>
+      <c r="E281">
+        <v>10.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Sep 9 CMJ data
Practice session, all 28 roster players, prior 280 rows untouched. Ava
Heil, Emma Blakely and Juliet Thrapp have no jumps recorded and carry
through as blanks rather than zeros.

Session quality is normal -- median trial spread 0.40 cm, matching the
season -- with one exception: Molly Bachman's 15.2/13.1 pair is a 2.1 cm
spread, 3.8 SD against the season's trial-to-trial noise. Left as
recorded, since five comparable spreads already sit in the season and
nothing marks this one as the bad trial.

The derived noise floor moves 0.65 -> 0.67 cm, since it recomputes from
every paired trial including today's.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/WSOC_CMJ_Season.xlsx
+++ b/sample_data/WSOC_CMJ_Season.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahc\Desktop\PLNU_WSOC_SS\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39A234CB-3017-4C32-BC00-18EA622856BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A603B48E-4C47-483E-8870-4BAC88E821F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="33">
   <si>
     <t>Date</t>
   </si>
@@ -498,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E281"/>
+  <dimension ref="A1:E309"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -5054,6 +5054,464 @@
         <v>10.5</v>
       </c>
     </row>
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A282" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B282" t="b">
+        <v>0</v>
+      </c>
+      <c r="C282" t="s">
+        <v>5</v>
+      </c>
+      <c r="D282">
+        <v>14.7</v>
+      </c>
+      <c r="E282">
+        <v>14.7</v>
+      </c>
+    </row>
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A283" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B283" t="b">
+        <v>0</v>
+      </c>
+      <c r="C283" t="s">
+        <v>6</v>
+      </c>
+      <c r="D283">
+        <v>13.5</v>
+      </c>
+      <c r="E283">
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A284" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B284" t="b">
+        <v>0</v>
+      </c>
+      <c r="C284" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A285" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B285" t="b">
+        <v>0</v>
+      </c>
+      <c r="C285" t="s">
+        <v>8</v>
+      </c>
+      <c r="D285">
+        <v>13.7</v>
+      </c>
+      <c r="E285">
+        <v>13.7</v>
+      </c>
+    </row>
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A286" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B286" t="b">
+        <v>0</v>
+      </c>
+      <c r="C286" t="s">
+        <v>9</v>
+      </c>
+      <c r="D286">
+        <v>12.5</v>
+      </c>
+      <c r="E286">
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A287" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B287" t="b">
+        <v>0</v>
+      </c>
+      <c r="C287" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A288" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B288" t="b">
+        <v>0</v>
+      </c>
+      <c r="C288" t="s">
+        <v>11</v>
+      </c>
+      <c r="D288">
+        <v>15.5</v>
+      </c>
+      <c r="E288">
+        <v>15.3</v>
+      </c>
+    </row>
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A289" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B289" t="b">
+        <v>0</v>
+      </c>
+      <c r="C289" t="s">
+        <v>12</v>
+      </c>
+      <c r="D289">
+        <v>9.9</v>
+      </c>
+      <c r="E289">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A290" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B290" t="b">
+        <v>0</v>
+      </c>
+      <c r="C290" t="s">
+        <v>13</v>
+      </c>
+      <c r="D290">
+        <v>14.7</v>
+      </c>
+      <c r="E290">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A291" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B291" t="b">
+        <v>0</v>
+      </c>
+      <c r="C291" t="s">
+        <v>14</v>
+      </c>
+      <c r="D291">
+        <v>13.5</v>
+      </c>
+      <c r="E291">
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A292" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B292" t="b">
+        <v>0</v>
+      </c>
+      <c r="C292" t="s">
+        <v>15</v>
+      </c>
+      <c r="D292">
+        <v>13.6</v>
+      </c>
+      <c r="E292">
+        <v>14.2</v>
+      </c>
+    </row>
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A293" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B293" t="b">
+        <v>0</v>
+      </c>
+      <c r="C293" t="s">
+        <v>16</v>
+      </c>
+      <c r="D293">
+        <v>13.8</v>
+      </c>
+      <c r="E293">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A294" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B294" t="b">
+        <v>0</v>
+      </c>
+      <c r="C294" t="s">
+        <v>17</v>
+      </c>
+      <c r="D294">
+        <v>13.9</v>
+      </c>
+      <c r="E294">
+        <v>12.9</v>
+      </c>
+    </row>
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A295" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B295" t="b">
+        <v>0</v>
+      </c>
+      <c r="C295" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A296" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B296" t="b">
+        <v>0</v>
+      </c>
+      <c r="C296" t="s">
+        <v>19</v>
+      </c>
+      <c r="D296">
+        <v>12.2</v>
+      </c>
+      <c r="E296">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A297" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B297" t="b">
+        <v>0</v>
+      </c>
+      <c r="C297" t="s">
+        <v>20</v>
+      </c>
+      <c r="D297">
+        <v>12.7</v>
+      </c>
+      <c r="E297">
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A298" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B298" t="b">
+        <v>0</v>
+      </c>
+      <c r="C298" t="s">
+        <v>21</v>
+      </c>
+      <c r="D298">
+        <v>15.4</v>
+      </c>
+      <c r="E298">
+        <v>15.8</v>
+      </c>
+    </row>
+    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A299" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B299" t="b">
+        <v>0</v>
+      </c>
+      <c r="C299" t="s">
+        <v>22</v>
+      </c>
+      <c r="D299">
+        <v>10.9</v>
+      </c>
+      <c r="E299">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A300" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B300" t="b">
+        <v>0</v>
+      </c>
+      <c r="C300" t="s">
+        <v>23</v>
+      </c>
+      <c r="D300">
+        <v>15.7</v>
+      </c>
+      <c r="E300">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A301" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B301" t="b">
+        <v>0</v>
+      </c>
+      <c r="C301" t="s">
+        <v>24</v>
+      </c>
+      <c r="D301">
+        <v>13.5</v>
+      </c>
+      <c r="E301">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A302" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B302" t="b">
+        <v>0</v>
+      </c>
+      <c r="C302" t="s">
+        <v>25</v>
+      </c>
+      <c r="D302">
+        <v>9.5</v>
+      </c>
+      <c r="E302">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A303" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B303" t="b">
+        <v>0</v>
+      </c>
+      <c r="C303" t="s">
+        <v>26</v>
+      </c>
+      <c r="D303">
+        <v>13.2</v>
+      </c>
+      <c r="E303">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A304" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B304" t="b">
+        <v>0</v>
+      </c>
+      <c r="C304" t="s">
+        <v>27</v>
+      </c>
+      <c r="D304">
+        <v>15.2</v>
+      </c>
+      <c r="E304">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A305" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B305" t="b">
+        <v>0</v>
+      </c>
+      <c r="C305" t="s">
+        <v>28</v>
+      </c>
+      <c r="D305">
+        <v>15.7</v>
+      </c>
+      <c r="E305">
+        <v>15.7</v>
+      </c>
+    </row>
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A306" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B306" t="b">
+        <v>0</v>
+      </c>
+      <c r="C306" t="s">
+        <v>29</v>
+      </c>
+      <c r="D306">
+        <v>13.7</v>
+      </c>
+      <c r="E306">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A307" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B307" t="b">
+        <v>0</v>
+      </c>
+      <c r="C307" t="s">
+        <v>30</v>
+      </c>
+      <c r="D307">
+        <v>13</v>
+      </c>
+      <c r="E307">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A308" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B308" t="b">
+        <v>0</v>
+      </c>
+      <c r="C308" t="s">
+        <v>31</v>
+      </c>
+      <c r="D308">
+        <v>12.8</v>
+      </c>
+      <c r="E308">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A309" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B309" t="b">
+        <v>0</v>
+      </c>
+      <c r="C309" t="s">
+        <v>32</v>
+      </c>
+      <c r="D309">
+        <v>12.4</v>
+      </c>
+      <c r="E309">
+        <v>11.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Sep 10 CMJ data
Match day vs LA, all 28 roster players, prior 308 rows untouched. The squad
came late from a film session, so only 18 jumped; the other ten carry through
as blanks rather than zeros. Four of the ten -- Bachman, Bisset, Masinter and
Naftzger -- started the match.

Session quality is normal: median trial spread 0.35 cm against 0.40 for the
season. The widest pair is Leah Uezato's 10.8/12.0, 2.1 SD against the
season's trial-to-trial noise, with eleven comparable spreads already in the
sheet, so it is left as recorded. The derived noise floor moves 0.67 -> 0.66 cm.

Kody McKinney comes off the watchlist: his jump is back to 13.45 cm from
12.45, above his own median, leaving him "Load only".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/WSOC_CMJ_Season.xlsx
+++ b/sample_data/WSOC_CMJ_Season.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahc\Desktop\PLNU_WSOC_SS\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A603B48E-4C47-483E-8870-4BAC88E821F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{162F6524-D0E2-4F23-B3FC-672667CE67ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="33">
   <si>
     <t>Date</t>
   </si>
@@ -498,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E309"/>
+  <dimension ref="A1:E337"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -5512,6 +5512,422 @@
         <v>11.6</v>
       </c>
     </row>
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A310" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B310" t="b">
+        <v>1</v>
+      </c>
+      <c r="C310" t="s">
+        <v>5</v>
+      </c>
+      <c r="D310">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="E310">
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A311" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B311" t="b">
+        <v>1</v>
+      </c>
+      <c r="C311" t="s">
+        <v>6</v>
+      </c>
+      <c r="D311">
+        <v>13.3</v>
+      </c>
+      <c r="E311">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A312" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B312" t="b">
+        <v>1</v>
+      </c>
+      <c r="C312" t="s">
+        <v>7</v>
+      </c>
+      <c r="D312">
+        <v>14.8</v>
+      </c>
+      <c r="E312">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A313" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B313" t="b">
+        <v>1</v>
+      </c>
+      <c r="C313" t="s">
+        <v>8</v>
+      </c>
+      <c r="D313">
+        <v>13.7</v>
+      </c>
+      <c r="E313">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A314" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B314" t="b">
+        <v>1</v>
+      </c>
+      <c r="C314" t="s">
+        <v>9</v>
+      </c>
+      <c r="D314">
+        <v>11.2</v>
+      </c>
+      <c r="E314">
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A315" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B315" t="b">
+        <v>1</v>
+      </c>
+      <c r="C315" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A316" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B316" t="b">
+        <v>1</v>
+      </c>
+      <c r="C316" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A317" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B317" t="b">
+        <v>1</v>
+      </c>
+      <c r="C317" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A318" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B318" t="b">
+        <v>1</v>
+      </c>
+      <c r="C318" t="s">
+        <v>13</v>
+      </c>
+      <c r="D318">
+        <v>14.9</v>
+      </c>
+      <c r="E318">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A319" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B319" t="b">
+        <v>1</v>
+      </c>
+      <c r="C319" t="s">
+        <v>14</v>
+      </c>
+      <c r="D319">
+        <v>12.8</v>
+      </c>
+      <c r="E319">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A320" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B320" t="b">
+        <v>1</v>
+      </c>
+      <c r="C320" t="s">
+        <v>15</v>
+      </c>
+      <c r="D320">
+        <v>13.3</v>
+      </c>
+      <c r="E320">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A321" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B321" t="b">
+        <v>1</v>
+      </c>
+      <c r="C321" t="s">
+        <v>16</v>
+      </c>
+      <c r="D321">
+        <v>14</v>
+      </c>
+      <c r="E321">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A322" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B322" t="b">
+        <v>1</v>
+      </c>
+      <c r="C322" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A323" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B323" t="b">
+        <v>1</v>
+      </c>
+      <c r="C323" t="s">
+        <v>18</v>
+      </c>
+      <c r="D323">
+        <v>14.6</v>
+      </c>
+      <c r="E323">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A324" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B324" t="b">
+        <v>1</v>
+      </c>
+      <c r="C324" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A325" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B325" t="b">
+        <v>1</v>
+      </c>
+      <c r="C325" t="s">
+        <v>20</v>
+      </c>
+      <c r="D325">
+        <v>13.3</v>
+      </c>
+      <c r="E325">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A326" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B326" t="b">
+        <v>1</v>
+      </c>
+      <c r="C326" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A327" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B327" t="b">
+        <v>1</v>
+      </c>
+      <c r="C327" t="s">
+        <v>22</v>
+      </c>
+      <c r="D327">
+        <v>10.8</v>
+      </c>
+      <c r="E327">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A328" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B328" t="b">
+        <v>1</v>
+      </c>
+      <c r="C328" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A329" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B329" t="b">
+        <v>1</v>
+      </c>
+      <c r="C329" t="s">
+        <v>24</v>
+      </c>
+      <c r="D329">
+        <v>13.8</v>
+      </c>
+      <c r="E329">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A330" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B330" t="b">
+        <v>1</v>
+      </c>
+      <c r="C330" t="s">
+        <v>25</v>
+      </c>
+      <c r="D330">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="E330">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A331" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B331" t="b">
+        <v>1</v>
+      </c>
+      <c r="C331" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A332" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B332" t="b">
+        <v>1</v>
+      </c>
+      <c r="C332" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A333" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B333" t="b">
+        <v>1</v>
+      </c>
+      <c r="C333" t="s">
+        <v>28</v>
+      </c>
+      <c r="D333">
+        <v>17.3</v>
+      </c>
+      <c r="E333">
+        <v>16.600000000000001</v>
+      </c>
+    </row>
+    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A334" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B334" t="b">
+        <v>1</v>
+      </c>
+      <c r="C334" t="s">
+        <v>29</v>
+      </c>
+      <c r="D334">
+        <v>13.9</v>
+      </c>
+      <c r="E334">
+        <v>13.7</v>
+      </c>
+    </row>
+    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A335" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B335" t="b">
+        <v>1</v>
+      </c>
+      <c r="C335" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A336" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B336" t="b">
+        <v>1</v>
+      </c>
+      <c r="C336" t="s">
+        <v>31</v>
+      </c>
+      <c r="D336">
+        <v>12.1</v>
+      </c>
+      <c r="E336">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A337" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B337" t="b">
+        <v>1</v>
+      </c>
+      <c r="C337" t="s">
+        <v>32</v>
+      </c>
+      <c r="D337">
+        <v>11.3</v>
+      </c>
+      <c r="E337">
+        <v>11.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>